<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-11T12:34Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -536,23 +536,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -569,23 +573,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -597,24 +605,20 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -622,7 +626,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -634,32 +638,28 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -676,27 +676,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -713,12 +713,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -728,12 +728,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -750,27 +750,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -787,27 +787,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -824,12 +824,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -839,12 +839,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -861,27 +861,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -898,27 +898,27 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -950,12 +950,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -972,27 +972,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1009,27 +1009,27 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1046,27 +1046,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1083,27 +1083,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1120,27 +1120,27 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1172,12 +1172,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1194,12 +1194,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1209,12 +1209,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1246,12 +1246,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1268,12 +1268,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1283,12 +1283,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>에이지테크, AX</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1305,12 +1305,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1342,27 +1342,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1379,23 +1379,27 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1412,15 +1416,19 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>산업통상부</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -1428,7 +1436,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1445,33 +1453,99 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>광주정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G28"/>
+  <autoFilter ref="A1:G30"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -1500,6 +1574,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>